<commit_message>
Added 3 stages of T-Shirt size estimation from my WBS
</commit_message>
<xml_diff>
--- a/Estimation/Estimation_Test.xlsx
+++ b/Estimation/Estimation_Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\SkillsRepository\Estimation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA87E21C-452C-44BA-A4B9-4565EFEE0C6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE61CC79-0492-4F84-A7B5-D0A8FE9E494B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="53">
   <si>
     <t>На прикладі задач Technical Artist</t>
   </si>
@@ -87,9 +87,6 @@
     <t>16 – 32 hours</t>
   </si>
   <si>
-    <t>Stage 1</t>
-  </si>
-  <si>
     <t>Task Number</t>
   </si>
   <si>
@@ -115,13 +112,97 @@
   </si>
   <si>
     <t>Estimated Hours Range (example)</t>
+  </si>
+  <si>
+    <t>Overall Estimation Time:</t>
+  </si>
+  <si>
+    <t>Stage 2: Reskinning assets (UI, reels, symbols, bg, etc..)</t>
+  </si>
+  <si>
+    <t>Stage 1: Masterfile</t>
+  </si>
+  <si>
+    <t>Adjust correct resolution</t>
+  </si>
+  <si>
+    <t>Creating new assets</t>
+  </si>
+  <si>
+    <t>Adjust by Masterfile (resolution, color, filters, etc..)</t>
+  </si>
+  <si>
+    <t>Creating new animation</t>
+  </si>
+  <si>
+    <t>Correcting scale, naming, hierarchy</t>
+  </si>
+  <si>
+    <t>Animation, mask, weigh corrections</t>
+  </si>
+  <si>
+    <t>Export assets (.JSON, ,spine files)</t>
+  </si>
+  <si>
+    <t>2.1.1</t>
+  </si>
+  <si>
+    <t>2.2.1</t>
+  </si>
+  <si>
+    <t>2.2.2</t>
+  </si>
+  <si>
+    <t>2.3.1</t>
+  </si>
+  <si>
+    <t>2.3.2</t>
+  </si>
+  <si>
+    <t>2.3.3</t>
+  </si>
+  <si>
+    <t>Replace assets in works folder</t>
+  </si>
+  <si>
+    <t>Stage 3: Fonts reskin</t>
+  </si>
+  <si>
+    <t>Creating bitmap font sprite</t>
+  </si>
+  <si>
+    <t>Exporting sprite</t>
+  </si>
+  <si>
+    <t>Import to Shoebox (or similar tool)</t>
+  </si>
+  <si>
+    <t>Creating bitmap font and .xml</t>
+  </si>
+  <si>
+    <t>Renaming .ttf font</t>
+  </si>
+  <si>
+    <t>3.1.1</t>
+  </si>
+  <si>
+    <t>3.1.2</t>
+  </si>
+  <si>
+    <t>3.1.3</t>
+  </si>
+  <si>
+    <t>3.1.4</t>
+  </si>
+  <si>
+    <t>3.3.1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -162,6 +243,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="22"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -198,7 +294,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -208,6 +304,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -221,6 +320,33 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -523,164 +649,468 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BA3DA27-D97A-42F1-BEEC-9C03BA47D32A}">
-  <dimension ref="B4:K13"/>
+  <dimension ref="B3:K39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="6" width="19.85546875" customWidth="1"/>
-    <col min="10" max="10" width="11.140625" customWidth="1"/>
-    <col min="11" max="11" width="20.140625" customWidth="1"/>
-    <col min="12" max="12" width="15.5703125" customWidth="1"/>
-    <col min="13" max="13" width="17.85546875" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="10"/>
+    <col min="2" max="6" width="19.85546875" style="10" customWidth="1"/>
+    <col min="7" max="9" width="9.140625" style="10"/>
+    <col min="10" max="10" width="11.140625" style="10" customWidth="1"/>
+    <col min="11" max="11" width="20.140625" style="10" customWidth="1"/>
+    <col min="12" max="12" width="15.5703125" style="10" customWidth="1"/>
+    <col min="13" max="13" width="17.85546875" style="10" customWidth="1"/>
+    <col min="14" max="16384" width="9.140625" style="10"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
+    <row r="3" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+    </row>
+    <row r="4" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+    </row>
+    <row r="6" spans="2:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="B6" s="6" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="6" spans="2:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="B6" s="5" t="s">
+      <c r="C6" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="7">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C7" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="D7" s="8"/>
+      <c r="E7" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="F7" s="8">
+        <v>10</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="8"/>
+      <c r="E8" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" s="8">
         <v>2</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="E6" s="5" t="s">
+      <c r="J8" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="8"/>
+      <c r="E9" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="8">
         <v>4</v>
       </c>
-      <c r="F6" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="K6" s="5" t="s">
+      <c r="J9" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="K9" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="7">
+        <v>1.2</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="8"/>
+      <c r="E10" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" s="8">
+        <v>2</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="K10" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="7">
+        <v>1.3</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="8"/>
+      <c r="E11" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" s="8">
+        <v>1</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="5"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="7" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="6">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="7"/>
-      <c r="E7" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="F7" s="7">
-        <v>8</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="K7" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" s="7" t="s">
+      <c r="E12" s="3"/>
+      <c r="F12" s="4">
+        <f>SUM(F7:F11)</f>
         <v>19</v>
       </c>
-      <c r="D8" s="7"/>
-      <c r="E8" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F8" s="7">
-        <v>4</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="K8" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="7"/>
-      <c r="E9" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="F9" s="7">
-        <v>6</v>
-      </c>
-      <c r="J9" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="K9" s="7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="6">
-        <v>1.2</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D10" s="7"/>
-      <c r="E10" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="F10" s="7">
-        <v>12</v>
-      </c>
-      <c r="J10" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="K10" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="6">
-        <v>1.3</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="7"/>
-      <c r="E11" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F11" s="7">
-        <v>2</v>
-      </c>
-      <c r="J11" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="K11" s="7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="4"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="2"/>
     </row>
     <row r="13" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="4"/>
+      <c r="B13" s="5"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="3"/>
       <c r="F13" s="2"/>
     </row>
+    <row r="15" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+    </row>
+    <row r="16" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B18" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="7">
+        <v>2.1</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="D19" s="8"/>
+      <c r="E19" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="F19" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D20" s="8"/>
+      <c r="E20" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="F20" s="15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="7">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="D21" s="8"/>
+      <c r="E21" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" s="15">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="D22" s="8"/>
+      <c r="E22" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="F22" s="15">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" s="8"/>
+      <c r="E23" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F23" s="16">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D24" s="12"/>
+      <c r="E24" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="F24" s="17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D25" s="12"/>
+      <c r="E25" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="F25" s="17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" s="12"/>
+      <c r="E26" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="F26" s="17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="D27" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F27" s="14">
+        <f>SUM(F19:F26)</f>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B30" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C30" s="11"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="11"/>
+      <c r="F30" s="11"/>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B31" s="11"/>
+      <c r="C31" s="11"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="11"/>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B33" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="B34" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="D34" s="8"/>
+      <c r="E34" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F34" s="15">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B35" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C35" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D35" s="8"/>
+      <c r="E35" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F35" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="B36" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C36" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="D36" s="8"/>
+      <c r="E36" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F36" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="B37" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D37" s="8"/>
+      <c r="E37" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="F37" s="16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B38" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C38" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D38" s="12"/>
+      <c r="E38" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="F38" s="17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39" spans="2:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="D39" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F39" s="14">
+        <f>SUM(F34:F38)</f>
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B15:F16"/>
+    <mergeCell ref="B3:F4"/>
+    <mergeCell ref="B30:F31"/>
+  </mergeCells>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Created "Three point Estimation" sheet with same case of Estimation tasks
</commit_message>
<xml_diff>
--- a/Estimation/Estimation_Test.xlsx
+++ b/Estimation/Estimation_Test.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\SkillsRepository\Estimation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE61CC79-0492-4F84-A7B5-D0A8FE9E494B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCEA0AF2-3A68-420F-8187-97A0C6BF6A14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="WBS" sheetId="1" r:id="rId1"/>
-    <sheet name="T-Shirt" sheetId="3" r:id="rId2"/>
+    <sheet name="T-Shirt" sheetId="3" r:id="rId1"/>
+    <sheet name="Three point Estimation" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,12 +37,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="53">
-  <si>
-    <t>На прикладі задач Technical Artist</t>
-  </si>
-  <si>
-    <t>Project</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="74">
+  <si>
+    <t>Notes</t>
   </si>
   <si>
     <t>Task Name</t>
@@ -196,13 +193,136 @@
   </si>
   <si>
     <t>3.3.1</t>
+  </si>
+  <si>
+    <t>.JSON, .spine</t>
+  </si>
+  <si>
+    <t>Three-Point Estimation</t>
+  </si>
+  <si>
+    <r>
+      <t>• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF313131"/>
+        <rFont val="Sigma Sans"/>
+      </rPr>
+      <t>Optimistic</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF313131"/>
+        <rFont val="Sigma Sans"/>
+      </rPr>
+      <t> – the minimum possible time or cost.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF313131"/>
+        <rFont val="Sigma Sans"/>
+      </rPr>
+      <t>Pessimistic</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF313131"/>
+        <rFont val="Sigma Sans"/>
+      </rPr>
+      <t> – the maximum possible time or cost.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF313131"/>
+        <rFont val="Sigma Sans"/>
+      </rPr>
+      <t>Most Likely</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF313131"/>
+        <rFont val="Sigma Sans"/>
+      </rPr>
+      <t> – a realistic estimate that is most to be accurate.</t>
+    </r>
+  </si>
+  <si>
+    <t>• Expected Case = (O + 4 × ML + P) / 6.</t>
+  </si>
+  <si>
+    <t>Optimistic (O)</t>
+  </si>
+  <si>
+    <t>Most Likely (M)</t>
+  </si>
+  <si>
+    <t>Pessimistic (P)</t>
+  </si>
+  <si>
+    <t>TOTAL (Stage 1)</t>
+  </si>
+  <si>
+    <t>Correct naming and hierarchy</t>
+  </si>
+  <si>
+    <t>Adjust resolution and scale</t>
+  </si>
+  <si>
+    <t>Expected Est. (E) hours</t>
+  </si>
+  <si>
+    <t>Example:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optimistic: </t>
+  </si>
+  <si>
+    <t>Hours</t>
+  </si>
+  <si>
+    <t>Pessimistic:</t>
+  </si>
+  <si>
+    <t>Reskinning symbols and reels</t>
+  </si>
+  <si>
+    <t>May occur some problems with layots, spine files, export, resolution. Need scale fixes</t>
+  </si>
+  <si>
+    <t>Most likely:</t>
+  </si>
+  <si>
+    <t>May be minor fixes and predictable adjustments</t>
+  </si>
+  <si>
+    <t>Will be no problems and issues with .spine files and source files (animations, naming, etc..)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -212,15 +332,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -258,6 +369,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF313131"/>
+      <name val="Sigma Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF313131"/>
+      <name val="Sigma Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -267,7 +397,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -290,48 +420,87 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -339,7 +508,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -347,6 +516,36 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -627,360 +826,341 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="F2:G4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="2" spans="6:7" x14ac:dyDescent="0.25">
-      <c r="F2" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="6:7" x14ac:dyDescent="0.25">
-      <c r="G4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BA3DA27-D97A-42F1-BEEC-9C03BA47D32A}">
   <dimension ref="B3:K39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="10"/>
-    <col min="2" max="6" width="19.85546875" style="10" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="10"/>
-    <col min="10" max="10" width="11.140625" style="10" customWidth="1"/>
-    <col min="11" max="11" width="20.140625" style="10" customWidth="1"/>
-    <col min="12" max="12" width="15.5703125" style="10" customWidth="1"/>
-    <col min="13" max="13" width="17.85546875" style="10" customWidth="1"/>
-    <col min="14" max="16384" width="9.140625" style="10"/>
+    <col min="1" max="1" width="9.140625" style="9"/>
+    <col min="2" max="6" width="19.85546875" style="9" customWidth="1"/>
+    <col min="7" max="9" width="9.140625" style="9"/>
+    <col min="10" max="10" width="11.140625" style="9" customWidth="1"/>
+    <col min="11" max="11" width="20.140625" style="9" customWidth="1"/>
+    <col min="12" max="12" width="15.5703125" style="9" customWidth="1"/>
+    <col min="13" max="13" width="17.85546875" style="9" customWidth="1"/>
+    <col min="14" max="16384" width="9.140625" style="9"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
+      <c r="B3" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
     </row>
     <row r="4" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
     </row>
     <row r="6" spans="2:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="6">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C7" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D7" s="7"/>
+      <c r="E7" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="F7" s="7">
+        <v>10</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="7"/>
+      <c r="E8" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="F8" s="7">
         <v>2</v>
       </c>
-      <c r="D6" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E6" s="6" t="s">
+      <c r="J8" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="7"/>
+      <c r="E9" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="F9" s="7">
         <v>4</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="J9" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="J6" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="K6" s="6" t="s">
+      <c r="K9" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="6">
+        <v>1.2</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="7"/>
+      <c r="E10" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="F10" s="7">
+        <v>2</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="6">
+        <v>1.3</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="7"/>
+      <c r="E11" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" s="7">
+        <v>1</v>
+      </c>
+      <c r="J11" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="4"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="7">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="F7" s="8">
-        <v>10</v>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="K7" s="8" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="8"/>
-      <c r="E8" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="F8" s="8">
-        <v>2</v>
-      </c>
-      <c r="J8" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="K8" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" s="8"/>
-      <c r="E9" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="F9" s="8">
-        <v>4</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="K9" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="7">
-        <v>1.2</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10" s="8"/>
-      <c r="E10" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="F10" s="8">
-        <v>2</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="K10" s="8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="7">
-        <v>1.3</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="D11" s="8"/>
-      <c r="E11" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="F11" s="8">
-        <v>1</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="K11" s="8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="5"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="4">
+      <c r="E12" s="2"/>
+      <c r="F12" s="3">
         <f>SUM(F7:F11)</f>
         <v>19</v>
       </c>
     </row>
     <row r="13" spans="2:11" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="5"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="2"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="1"/>
     </row>
     <row r="15" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
+      <c r="B15" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
     </row>
     <row r="16" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B18" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C18" s="6" t="s">
+      <c r="B18" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="E18" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="F18" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F18" s="6" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="19" spans="2:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="7">
+      <c r="B19" s="6">
         <v>2.1</v>
       </c>
-      <c r="C19" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D19" s="8"/>
-      <c r="E19" s="9" t="s">
-        <v>7</v>
+      <c r="C19" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D19" s="7"/>
+      <c r="E19" s="8" t="s">
+        <v>6</v>
       </c>
       <c r="F19" s="15">
         <v>2</v>
       </c>
     </row>
     <row r="20" spans="2:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" s="8"/>
-      <c r="E20" s="9" t="s">
-        <v>7</v>
+      <c r="B20" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" s="7"/>
+      <c r="E20" s="8" t="s">
+        <v>6</v>
       </c>
       <c r="F20" s="15">
         <v>3</v>
       </c>
     </row>
     <row r="21" spans="2:6" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="7">
+      <c r="B21" s="6">
         <v>2.2000000000000002</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="D21" s="8"/>
-      <c r="E21" s="9" t="s">
-        <v>8</v>
+        <v>28</v>
+      </c>
+      <c r="D21" s="7"/>
+      <c r="E21" s="8" t="s">
+        <v>7</v>
       </c>
       <c r="F21" s="15">
         <v>12</v>
       </c>
     </row>
     <row r="22" spans="2:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D22" s="8"/>
-      <c r="E22" s="9" t="s">
-        <v>6</v>
+      <c r="B22" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D22" s="7"/>
+      <c r="E22" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="F22" s="15">
         <v>6</v>
       </c>
     </row>
     <row r="23" spans="2:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="C23" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="D23" s="8"/>
-      <c r="E23" s="9" t="s">
-        <v>8</v>
+      <c r="B23" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D23" s="7"/>
+      <c r="E23" s="8" t="s">
+        <v>7</v>
       </c>
       <c r="F23" s="16">
         <v>8</v>
       </c>
     </row>
     <row r="24" spans="2:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="D24" s="12"/>
-      <c r="E24" s="9" t="s">
-        <v>6</v>
+      <c r="B24" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="D24" s="11"/>
+      <c r="E24" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="F24" s="17">
         <v>4</v>
       </c>
     </row>
     <row r="25" spans="2:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="D25" s="12"/>
-      <c r="E25" s="9" t="s">
-        <v>6</v>
+      <c r="B25" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="D25" s="11"/>
+      <c r="E25" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="F25" s="17">
         <v>4</v>
       </c>
     </row>
     <row r="26" spans="2:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="D26" s="12"/>
-      <c r="E26" s="9" t="s">
-        <v>7</v>
+      <c r="B26" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>6</v>
       </c>
       <c r="F26" s="17">
         <v>2</v>
       </c>
     </row>
     <row r="27" spans="2:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="D27" s="2" t="s">
-        <v>25</v>
+      <c r="D27" s="1" t="s">
+        <v>24</v>
       </c>
       <c r="F27" s="14">
         <f>SUM(F19:F26)</f>
@@ -988,116 +1168,116 @@
       </c>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B30" s="11" t="s">
+      <c r="B30" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10"/>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B33" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="B34" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C34" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="11"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="11"/>
-    </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B31" s="11"/>
-      <c r="C31" s="11"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="11"/>
-    </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B33" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="34" spans="2:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="B34" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C34" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="D34" s="8"/>
-      <c r="E34" s="9" t="s">
-        <v>8</v>
+      <c r="D34" s="7"/>
+      <c r="E34" s="8" t="s">
+        <v>7</v>
       </c>
       <c r="F34" s="15">
         <v>8</v>
       </c>
     </row>
     <row r="35" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B35" s="7" t="s">
-        <v>49</v>
+      <c r="B35" s="6" t="s">
+        <v>48</v>
       </c>
       <c r="C35" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="D35" s="8"/>
-      <c r="E35" s="9" t="s">
-        <v>9</v>
+        <v>43</v>
+      </c>
+      <c r="D35" s="7"/>
+      <c r="E35" s="8" t="s">
+        <v>8</v>
       </c>
       <c r="F35" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="36" spans="2:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="B36" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C36" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D36" s="8"/>
-      <c r="E36" s="9" t="s">
-        <v>9</v>
+      <c r="B36" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C36" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D36" s="7"/>
+      <c r="E36" s="8" t="s">
+        <v>8</v>
       </c>
       <c r="F36" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="37" spans="2:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="B37" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="C37" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="D37" s="8"/>
-      <c r="E37" s="9" t="s">
-        <v>7</v>
+      <c r="B37" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C37" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="D37" s="7"/>
+      <c r="E37" s="8" t="s">
+        <v>6</v>
       </c>
       <c r="F37" s="16">
         <v>2</v>
       </c>
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B38" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="C38" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="D38" s="12"/>
-      <c r="E38" s="9" t="s">
-        <v>6</v>
+      <c r="B38" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C38" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D38" s="11"/>
+      <c r="E38" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="F38" s="17">
         <v>4</v>
       </c>
     </row>
     <row r="39" spans="2:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="D39" s="2" t="s">
-        <v>25</v>
+      <c r="D39" s="1" t="s">
+        <v>24</v>
       </c>
       <c r="F39" s="14">
         <f>SUM(F34:F38)</f>
@@ -1110,7 +1290,248 @@
     <mergeCell ref="B3:F4"/>
     <mergeCell ref="B30:F31"/>
   </mergeCells>
-  <phoneticPr fontId="6" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D97CD3DD-2994-4D3B-91F4-7AF0F4C5171A}">
+  <dimension ref="B3:S17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="7" width="16" customWidth="1"/>
+    <col min="9" max="11" width="13.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:19" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="J3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="2:19" ht="45" x14ac:dyDescent="0.25">
+      <c r="I4" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="J4" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="K4" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="L4" s="29"/>
+      <c r="M4" s="29"/>
+      <c r="N4" s="29"/>
+      <c r="O4" s="29"/>
+      <c r="P4" s="29"/>
+      <c r="Q4" s="29"/>
+      <c r="R4" s="29"/>
+      <c r="S4" s="30"/>
+    </row>
+    <row r="5" spans="2:19" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="B5" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="I5" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="J5" s="26">
+        <v>6</v>
+      </c>
+      <c r="K5" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="L5" s="27"/>
+      <c r="M5" s="27"/>
+      <c r="N5" s="27"/>
+      <c r="O5" s="27"/>
+      <c r="P5" s="27"/>
+      <c r="Q5" s="27"/>
+      <c r="R5" s="27"/>
+      <c r="S5" s="27"/>
+    </row>
+    <row r="6" spans="2:19" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="B6" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="I6" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="J6" s="26">
+        <v>10</v>
+      </c>
+      <c r="K6" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="L6" s="27"/>
+      <c r="M6" s="27"/>
+      <c r="N6" s="27"/>
+      <c r="O6" s="27"/>
+      <c r="P6" s="27"/>
+      <c r="Q6" s="27"/>
+      <c r="R6" s="27"/>
+      <c r="S6" s="27"/>
+    </row>
+    <row r="7" spans="2:19" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="B7" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="I7" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="J7" s="26">
+        <v>8</v>
+      </c>
+      <c r="K7" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="L7" s="27"/>
+      <c r="M7" s="27"/>
+      <c r="N7" s="27"/>
+      <c r="O7" s="27"/>
+      <c r="P7" s="27"/>
+      <c r="Q7" s="27"/>
+      <c r="R7" s="27"/>
+      <c r="S7" s="27"/>
+    </row>
+    <row r="9" spans="2:19" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="C9" s="19" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="2:19" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C11" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="2:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="C12" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="7">
+        <v>8</v>
+      </c>
+      <c r="E12" s="7">
+        <v>10</v>
+      </c>
+      <c r="F12" s="7">
+        <v>14</v>
+      </c>
+      <c r="G12" s="22">
+        <f>(D12+4*E12+F12)/6</f>
+        <v>10.333333333333334</v>
+      </c>
+    </row>
+    <row r="13" spans="2:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="C13" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="D13" s="7">
+        <v>1</v>
+      </c>
+      <c r="E13" s="7">
+        <v>2</v>
+      </c>
+      <c r="F13" s="7">
+        <v>3</v>
+      </c>
+      <c r="G13" s="22">
+        <f>(D13+4*E13+F13)/6</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="2:19" ht="45" x14ac:dyDescent="0.25">
+      <c r="C14" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D14" s="7">
+        <v>3</v>
+      </c>
+      <c r="E14" s="7">
+        <v>4</v>
+      </c>
+      <c r="F14" s="7">
+        <v>6</v>
+      </c>
+      <c r="G14" s="22">
+        <f t="shared" ref="G13:G15" si="0">(D14+4*E14+F14)/6</f>
+        <v>4.166666666666667</v>
+      </c>
+    </row>
+    <row r="15" spans="2:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="C15" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" s="7">
+        <v>1</v>
+      </c>
+      <c r="E15" s="7">
+        <v>2</v>
+      </c>
+      <c r="F15" s="7">
+        <v>4</v>
+      </c>
+      <c r="G15" s="22">
+        <f>(D15+4*E15+F15)/6</f>
+        <v>2.1666666666666665</v>
+      </c>
+    </row>
+    <row r="16" spans="2:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="C16" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="E16" s="7">
+        <v>1</v>
+      </c>
+      <c r="F16" s="7">
+        <v>2</v>
+      </c>
+      <c r="G16" s="22">
+        <f>(D16+4*E16+F16)/6</f>
+        <v>1.0833333333333333</v>
+      </c>
+    </row>
+    <row r="17" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C17" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="23">
+        <f>SUM(G12:G16)</f>
+        <v>19.75</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="K7:S7"/>
+    <mergeCell ref="K4:S4"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="K5:S5"/>
+    <mergeCell ref="K6:S6"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Completed "Three point Estimation" sheet
</commit_message>
<xml_diff>
--- a/Estimation/Estimation_Test.xlsx
+++ b/Estimation/Estimation_Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\SkillsRepository\Estimation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCEA0AF2-3A68-420F-8187-97A0C6BF6A14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31C8D2DC-A0A1-434F-930E-C4E26CF4DF5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="81">
   <si>
     <t>Notes</t>
   </si>
@@ -315,7 +315,28 @@
     <t>May be minor fixes and predictable adjustments</t>
   </si>
   <si>
-    <t>Will be no problems and issues with .spine files and source files (animations, naming, etc..)</t>
+    <t>Will be no issues with .spine files and source files (animations, naming, etc..)</t>
+  </si>
+  <si>
+    <t>Animation, mask, weight corrections</t>
+  </si>
+  <si>
+    <t>Export assets (.JSON, .spine)</t>
+  </si>
+  <si>
+    <t>TOTAL (Stage 2)</t>
+  </si>
+  <si>
+    <t>Adjust by Masterfile</t>
+  </si>
+  <si>
+    <t>Adjust resolution</t>
+  </si>
+  <si>
+    <t>Import to Shoebox</t>
+  </si>
+  <si>
+    <t>TOTAL (Stage 3)</t>
   </si>
 </sst>
 </file>
@@ -461,7 +482,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -546,6 +567,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1297,7 +1321,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D97CD3DD-2994-4D3B-91F4-7AF0F4C5171A}">
-  <dimension ref="B3:S17"/>
+  <dimension ref="B3:S40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="7" width="16" customWidth="1"/>
@@ -1523,6 +1547,304 @@
         <f>SUM(G12:G16)</f>
         <v>19.75</v>
       </c>
+    </row>
+    <row r="20" spans="3:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="C20" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="3:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="C21" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" s="7">
+        <v>1</v>
+      </c>
+      <c r="E21" s="7">
+        <v>2</v>
+      </c>
+      <c r="F21" s="7">
+        <v>4</v>
+      </c>
+      <c r="G21" s="22">
+        <f>(D21+4*E21+F21)/6</f>
+        <v>2.1666666666666665</v>
+      </c>
+    </row>
+    <row r="22" spans="3:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="C22" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D22" s="7">
+        <v>2</v>
+      </c>
+      <c r="E22" s="7">
+        <v>3</v>
+      </c>
+      <c r="F22" s="7">
+        <v>5</v>
+      </c>
+      <c r="G22" s="22">
+        <f>(D22+4*E22+F22)/6</f>
+        <v>3.1666666666666665</v>
+      </c>
+    </row>
+    <row r="23" spans="3:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="C23" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D23" s="7">
+        <v>10</v>
+      </c>
+      <c r="E23" s="7">
+        <v>12</v>
+      </c>
+      <c r="F23" s="7">
+        <v>16</v>
+      </c>
+      <c r="G23" s="22">
+        <f t="shared" ref="G23" si="1">(D23+4*E23+F23)/6</f>
+        <v>12.333333333333334</v>
+      </c>
+    </row>
+    <row r="24" spans="3:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="C24" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="D24" s="7">
+        <v>4</v>
+      </c>
+      <c r="E24" s="7">
+        <v>6</v>
+      </c>
+      <c r="F24" s="7">
+        <v>9</v>
+      </c>
+      <c r="G24" s="22">
+        <f>(D24+4*E24+F24)/6</f>
+        <v>6.166666666666667</v>
+      </c>
+    </row>
+    <row r="25" spans="3:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="C25" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D25" s="7">
+        <v>6</v>
+      </c>
+      <c r="E25" s="7">
+        <v>8</v>
+      </c>
+      <c r="F25" s="7">
+        <v>12</v>
+      </c>
+      <c r="G25" s="22">
+        <f>(D25+4*E25+F25)/6</f>
+        <v>8.3333333333333339</v>
+      </c>
+    </row>
+    <row r="26" spans="3:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="C26" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D26" s="7">
+        <v>3</v>
+      </c>
+      <c r="E26" s="7">
+        <v>4</v>
+      </c>
+      <c r="F26" s="7">
+        <v>6</v>
+      </c>
+      <c r="G26" s="22">
+        <f>(D26+4*E26+F26)/6</f>
+        <v>4.166666666666667</v>
+      </c>
+    </row>
+    <row r="27" spans="3:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="C27" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="D27" s="7">
+        <v>3</v>
+      </c>
+      <c r="E27" s="7">
+        <v>4</v>
+      </c>
+      <c r="F27" s="7">
+        <v>6</v>
+      </c>
+      <c r="G27" s="22">
+        <f>(D27+4*E27+F27)/6</f>
+        <v>4.166666666666667</v>
+      </c>
+    </row>
+    <row r="28" spans="3:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="C28" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="D28" s="7">
+        <v>1</v>
+      </c>
+      <c r="E28" s="7">
+        <v>2</v>
+      </c>
+      <c r="F28" s="7">
+        <v>3</v>
+      </c>
+      <c r="G28" s="22">
+        <f t="shared" ref="G28" si="2">(D28+4*E28+F28)/6</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C29" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7"/>
+      <c r="G29" s="23">
+        <f>SUM(G21:G28)</f>
+        <v>42.5</v>
+      </c>
+    </row>
+    <row r="32" spans="3:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="C32" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="33" spans="3:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="C33" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D33" s="7">
+        <v>6</v>
+      </c>
+      <c r="E33" s="7">
+        <v>8</v>
+      </c>
+      <c r="F33" s="7">
+        <v>12</v>
+      </c>
+      <c r="G33" s="22">
+        <f>(D33+4*E33+F33)/6</f>
+        <v>8.3333333333333339</v>
+      </c>
+    </row>
+    <row r="34" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C34" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D34" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="E34" s="7">
+        <v>1</v>
+      </c>
+      <c r="F34" s="7">
+        <v>2</v>
+      </c>
+      <c r="G34" s="22">
+        <f>(D34+4*E34+F34)/6</f>
+        <v>1.0833333333333333</v>
+      </c>
+    </row>
+    <row r="35" spans="3:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="C35" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D35" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="E35" s="7">
+        <v>1</v>
+      </c>
+      <c r="F35" s="7">
+        <v>2</v>
+      </c>
+      <c r="G35" s="22">
+        <f t="shared" ref="G35" si="3">(D35+4*E35+F35)/6</f>
+        <v>1.0833333333333333</v>
+      </c>
+    </row>
+    <row r="36" spans="3:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="C36" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D36" s="7">
+        <v>1.5</v>
+      </c>
+      <c r="E36" s="7">
+        <v>2</v>
+      </c>
+      <c r="F36" s="7">
+        <v>3</v>
+      </c>
+      <c r="G36" s="22">
+        <f>(D36+4*E36+F36)/6</f>
+        <v>2.0833333333333335</v>
+      </c>
+    </row>
+    <row r="37" spans="3:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="C37" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D37" s="7">
+        <v>3</v>
+      </c>
+      <c r="E37" s="7">
+        <v>4</v>
+      </c>
+      <c r="F37" s="7">
+        <v>6</v>
+      </c>
+      <c r="G37" s="22">
+        <f>(D37+4*E37+F37)/6</f>
+        <v>4.166666666666667</v>
+      </c>
+    </row>
+    <row r="38" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C38" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="D38" s="7"/>
+      <c r="E38" s="7"/>
+      <c r="F38" s="7"/>
+      <c r="G38" s="23">
+        <f>SUM(G33:G37)</f>
+        <v>16.750000000000004</v>
+      </c>
+    </row>
+    <row r="39" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="G39" s="31"/>
+    </row>
+    <row r="40" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="G40" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
Added "Planning Poker" sheet and Parametric Estimation
</commit_message>
<xml_diff>
--- a/Estimation/Estimation_Test.xlsx
+++ b/Estimation/Estimation_Test.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\SkillsRepository\Estimation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31C8D2DC-A0A1-434F-930E-C4E26CF4DF5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86906610-7FE5-4AB2-8482-7A297CD0D217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T-Shirt" sheetId="3" r:id="rId1"/>
     <sheet name="Three point Estimation" sheetId="4" r:id="rId2"/>
+    <sheet name="Parametric Estimation" sheetId="5" r:id="rId3"/>
+    <sheet name="Planning Poker" sheetId="6" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="110">
   <si>
     <t>Notes</t>
   </si>
@@ -338,12 +340,99 @@
   <si>
     <t>TOTAL (Stage 3)</t>
   </si>
+  <si>
+    <t>Parametric Estimation</t>
+  </si>
+  <si>
+    <t>for example, 1 asset takes 5 minutes to export (includes naming, format check, organizing)</t>
+  </si>
+  <si>
+    <t>and there are 24 assets in total</t>
+  </si>
+  <si>
+    <t>Time per asset</t>
+  </si>
+  <si>
+    <t>5 min</t>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Total assets</t>
+  </si>
+  <si>
+    <t>Total time: 5 × 24</t>
+  </si>
+  <si>
+    <t>120 min = 2 hours</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Expert Judgement: Planning Poker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planning Poker is a gamified group estimation technique adapted from the Delphi method. </t>
+  </si>
+  <si>
+    <t>It helps teams reach a consensus when estimating tasks and user stories, making the process more interactive and engaging.</t>
+  </si>
+  <si>
+    <t>All experts gather in one room.</t>
+  </si>
+  <si>
+    <t>Each participant is given a set of cards with numbers from the Fibonacci sequence (e.g., 1, 2, 3, 5, 8, 13, etc.).</t>
+  </si>
+  <si>
+    <t>Example</t>
+  </si>
+  <si>
+    <t>Task: Creating bitmap font</t>
+  </si>
+  <si>
+    <t>I've done this many times - just a sprite and a Shoebox</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>5 hours</t>
+  </si>
+  <si>
+    <t>8 hours</t>
+  </si>
+  <si>
+    <t>3 hours</t>
+  </si>
+  <si>
+    <t>Dev1</t>
+  </si>
+  <si>
+    <t>Dev2</t>
+  </si>
+  <si>
+    <t>Dev3</t>
+  </si>
+  <si>
+    <t>I've done similar fonts before; it usually takes for me 4-5 hours.</t>
+  </si>
+  <si>
+    <t>There's can be issues with custom format + need scaling and styling adjustments</t>
+  </si>
+  <si>
+    <t>Final agreed estimate: 5 hours, medium risk, includes possible issues solving</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -402,8 +491,53 @@
       <name val="Sigma Sans"/>
     </font>
     <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="17"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF313131"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -482,7 +616,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -539,7 +673,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -551,6 +685,7 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -570,6 +705,53 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1343,86 +1525,86 @@
       <c r="I4" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="J4" s="24" t="s">
+      <c r="J4" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="K4" s="28" t="s">
+      <c r="K4" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="L4" s="29"/>
-      <c r="M4" s="29"/>
-      <c r="N4" s="29"/>
-      <c r="O4" s="29"/>
-      <c r="P4" s="29"/>
-      <c r="Q4" s="29"/>
-      <c r="R4" s="29"/>
-      <c r="S4" s="30"/>
+      <c r="L4" s="30"/>
+      <c r="M4" s="30"/>
+      <c r="N4" s="30"/>
+      <c r="O4" s="30"/>
+      <c r="P4" s="30"/>
+      <c r="Q4" s="30"/>
+      <c r="R4" s="30"/>
+      <c r="S4" s="31"/>
     </row>
     <row r="5" spans="2:19" ht="17.25" x14ac:dyDescent="0.3">
       <c r="B5" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="I5" s="25" t="s">
+      <c r="I5" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="J5" s="26">
+      <c r="J5" s="27">
         <v>6</v>
       </c>
-      <c r="K5" s="27" t="s">
+      <c r="K5" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="L5" s="27"/>
-      <c r="M5" s="27"/>
-      <c r="N5" s="27"/>
-      <c r="O5" s="27"/>
-      <c r="P5" s="27"/>
-      <c r="Q5" s="27"/>
-      <c r="R5" s="27"/>
-      <c r="S5" s="27"/>
+      <c r="L5" s="28"/>
+      <c r="M5" s="28"/>
+      <c r="N5" s="28"/>
+      <c r="O5" s="28"/>
+      <c r="P5" s="28"/>
+      <c r="Q5" s="28"/>
+      <c r="R5" s="28"/>
+      <c r="S5" s="28"/>
     </row>
     <row r="6" spans="2:19" ht="17.25" x14ac:dyDescent="0.3">
       <c r="B6" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="I6" s="25" t="s">
+      <c r="I6" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="J6" s="26">
+      <c r="J6" s="27">
         <v>10</v>
       </c>
-      <c r="K6" s="27" t="s">
+      <c r="K6" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="L6" s="27"/>
-      <c r="M6" s="27"/>
-      <c r="N6" s="27"/>
-      <c r="O6" s="27"/>
-      <c r="P6" s="27"/>
-      <c r="Q6" s="27"/>
-      <c r="R6" s="27"/>
-      <c r="S6" s="27"/>
+      <c r="L6" s="28"/>
+      <c r="M6" s="28"/>
+      <c r="N6" s="28"/>
+      <c r="O6" s="28"/>
+      <c r="P6" s="28"/>
+      <c r="Q6" s="28"/>
+      <c r="R6" s="28"/>
+      <c r="S6" s="28"/>
     </row>
     <row r="7" spans="2:19" ht="17.25" x14ac:dyDescent="0.3">
       <c r="B7" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="I7" s="25" t="s">
+      <c r="I7" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="J7" s="26">
+      <c r="J7" s="27">
         <v>8</v>
       </c>
-      <c r="K7" s="27" t="s">
+      <c r="K7" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="L7" s="27"/>
-      <c r="M7" s="27"/>
-      <c r="N7" s="27"/>
-      <c r="O7" s="27"/>
-      <c r="P7" s="27"/>
-      <c r="Q7" s="27"/>
-      <c r="R7" s="27"/>
-      <c r="S7" s="27"/>
+      <c r="L7" s="28"/>
+      <c r="M7" s="28"/>
+      <c r="N7" s="28"/>
+      <c r="O7" s="28"/>
+      <c r="P7" s="28"/>
+      <c r="Q7" s="28"/>
+      <c r="R7" s="28"/>
+      <c r="S7" s="28"/>
     </row>
     <row r="9" spans="2:19" ht="17.25" x14ac:dyDescent="0.3">
       <c r="C9" s="19" t="s">
@@ -1841,10 +2023,10 @@
       </c>
     </row>
     <row r="39" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="G39" s="31"/>
+      <c r="G39" s="32"/>
     </row>
     <row r="40" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="G40" s="31"/>
+      <c r="G40" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1856,4 +2038,232 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2A0065E-4D3F-4550-8F31-85FFBED1E6CB}">
+  <dimension ref="C3:F8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="42.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="3:6" ht="21" x14ac:dyDescent="0.35">
+      <c r="C3" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+    </row>
+    <row r="4" spans="3:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C4" s="38" t="s">
+        <v>86</v>
+      </c>
+      <c r="D4" s="39" t="s">
+        <v>87</v>
+      </c>
+      <c r="E4" s="40"/>
+      <c r="F4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C5" s="33" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="29" t="s">
+        <v>91</v>
+      </c>
+      <c r="E5" s="31"/>
+      <c r="F5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C6" s="26" t="s">
+        <v>84</v>
+      </c>
+      <c r="D6" s="35" t="s">
+        <v>85</v>
+      </c>
+      <c r="E6" s="36"/>
+    </row>
+    <row r="7" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C7" s="26" t="s">
+        <v>88</v>
+      </c>
+      <c r="D7" s="35">
+        <v>24</v>
+      </c>
+      <c r="E7" s="36"/>
+    </row>
+    <row r="8" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C8" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="D8" s="34" t="s">
+        <v>90</v>
+      </c>
+      <c r="E8" s="34"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5E4CD89-6982-4E73-8AC7-7C0F51F5A6DD}">
+  <dimension ref="B4:K19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="3" width="9.140625" style="24"/>
+    <col min="4" max="4" width="11.7109375" style="24" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" style="24" customWidth="1"/>
+    <col min="6" max="10" width="9.140625" style="24"/>
+    <col min="11" max="11" width="39.140625" style="24" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="24"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="2:11" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="B4" s="41" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B5" s="42" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B6" s="24" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B8" s="51" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B9" s="51" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B13" s="43" t="s">
+        <v>97</v>
+      </c>
+      <c r="C13" s="43"/>
+      <c r="D13" s="43"/>
+      <c r="E13" s="43"/>
+      <c r="F13" s="43"/>
+      <c r="G13" s="43"/>
+      <c r="H13" s="43"/>
+      <c r="I13" s="43"/>
+      <c r="J13" s="43"/>
+      <c r="K13" s="43"/>
+    </row>
+    <row r="14" spans="2:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B14" s="44" t="s">
+        <v>98</v>
+      </c>
+      <c r="C14" s="44"/>
+      <c r="D14" s="44"/>
+      <c r="E14" s="45" t="s">
+        <v>87</v>
+      </c>
+      <c r="F14" s="46" t="s">
+        <v>100</v>
+      </c>
+      <c r="G14" s="46"/>
+      <c r="H14" s="46"/>
+      <c r="I14" s="46"/>
+      <c r="J14" s="46"/>
+      <c r="K14" s="46"/>
+    </row>
+    <row r="15" spans="2:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B15" s="47" t="s">
+        <v>104</v>
+      </c>
+      <c r="C15" s="47"/>
+      <c r="D15" s="47"/>
+      <c r="E15" s="48" t="s">
+        <v>101</v>
+      </c>
+      <c r="F15" s="49" t="s">
+        <v>107</v>
+      </c>
+      <c r="G15" s="49"/>
+      <c r="H15" s="49"/>
+      <c r="I15" s="49"/>
+      <c r="J15" s="49"/>
+      <c r="K15" s="49"/>
+    </row>
+    <row r="16" spans="2:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B16" s="47" t="s">
+        <v>105</v>
+      </c>
+      <c r="C16" s="47"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="48" t="s">
+        <v>102</v>
+      </c>
+      <c r="F16" s="49" t="s">
+        <v>108</v>
+      </c>
+      <c r="G16" s="49"/>
+      <c r="H16" s="49"/>
+      <c r="I16" s="49"/>
+      <c r="J16" s="49"/>
+      <c r="K16" s="49"/>
+    </row>
+    <row r="17" spans="2:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B17" s="47" t="s">
+        <v>106</v>
+      </c>
+      <c r="C17" s="47"/>
+      <c r="D17" s="47"/>
+      <c r="E17" s="48" t="s">
+        <v>103</v>
+      </c>
+      <c r="F17" s="49" t="s">
+        <v>99</v>
+      </c>
+      <c r="G17" s="49"/>
+      <c r="H17" s="49"/>
+      <c r="I17" s="49"/>
+      <c r="J17" s="49"/>
+      <c r="K17" s="49"/>
+    </row>
+    <row r="19" spans="2:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B19" s="24" t="s">
+        <v>109</v>
+      </c>
+      <c r="F19" s="50"/>
+      <c r="G19" s="50"/>
+      <c r="H19" s="50"/>
+      <c r="I19" s="50"/>
+      <c r="J19" s="50"/>
+      <c r="K19" s="50"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="F17:K17"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="F14:K14"/>
+    <mergeCell ref="F15:K15"/>
+    <mergeCell ref="F16:K16"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
some adjustments with fonts and metrics (L,M,XL)
</commit_message>
<xml_diff>
--- a/Estimation/Estimation_Test.xlsx
+++ b/Estimation/Estimation_Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\SkillsRepository\Estimation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86906610-7FE5-4AB2-8482-7A297CD0D217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B84DA6D7-9058-4A74-B417-E0DBCAFB6DEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T-Shirt" sheetId="3" r:id="rId1"/>
@@ -432,7 +432,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -514,13 +514,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="17"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color rgb="FF313131"/>
       <name val="Calibri"/>
@@ -538,6 +531,22 @@
     <font>
       <i/>
       <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -616,7 +625,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -645,72 +654,78 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -718,41 +733,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1047,20 +1043,20 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
     </row>
     <row r="4" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
+      <c r="B4" s="32"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
     </row>
     <row r="6" spans="2:11" ht="30" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
@@ -1094,7 +1090,7 @@
       </c>
       <c r="D7" s="7"/>
       <c r="E7" s="8" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F7" s="7">
         <v>10</v>
@@ -1210,20 +1206,20 @@
       <c r="F13" s="1"/>
     </row>
     <row r="15" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
+      <c r="C15" s="32"/>
+      <c r="D15" s="32"/>
+      <c r="E15" s="32"/>
+      <c r="F15" s="32"/>
     </row>
     <row r="16" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
+      <c r="B16" s="32"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="5" t="s">
@@ -1253,7 +1249,7 @@
       <c r="E19" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="F19" s="15">
+      <c r="F19" s="14">
         <v>2</v>
       </c>
     </row>
@@ -1268,7 +1264,7 @@
       <c r="E20" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="F20" s="15">
+      <c r="F20" s="14">
         <v>3</v>
       </c>
     </row>
@@ -1276,14 +1272,14 @@
       <c r="B21" s="6">
         <v>2.2000000000000002</v>
       </c>
-      <c r="C21" s="18" t="s">
+      <c r="C21" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D21" s="7"/>
       <c r="E21" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="F21" s="15">
+      <c r="F21" s="14">
         <v>12</v>
       </c>
     </row>
@@ -1291,14 +1287,14 @@
       <c r="B22" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="10" t="s">
         <v>29</v>
       </c>
       <c r="D22" s="7"/>
       <c r="E22" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="F22" s="15">
+      <c r="F22" s="14">
         <v>6</v>
       </c>
     </row>
@@ -1306,61 +1302,61 @@
       <c r="B23" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="10" t="s">
         <v>30</v>
       </c>
       <c r="D23" s="7"/>
       <c r="E23" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="F23" s="16">
+      <c r="F23" s="15">
         <v>8</v>
       </c>
     </row>
     <row r="24" spans="2:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="12" t="s">
+      <c r="B24" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D24" s="11"/>
+      <c r="D24" s="10"/>
       <c r="E24" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="F24" s="17">
+      <c r="F24" s="16">
         <v>4</v>
       </c>
     </row>
     <row r="25" spans="2:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D25" s="11"/>
+      <c r="D25" s="10"/>
       <c r="E25" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="F25" s="17">
+      <c r="F25" s="16">
         <v>4</v>
       </c>
     </row>
     <row r="26" spans="2:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="12" t="s">
+      <c r="B26" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C26" s="11" t="s">
+      <c r="C26" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="D26" s="11" t="s">
+      <c r="D26" s="10" t="s">
         <v>52</v>
       </c>
       <c r="E26" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="F26" s="17">
+      <c r="F26" s="16">
         <v>2</v>
       </c>
     </row>
@@ -1368,26 +1364,26 @@
       <c r="D27" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F27" s="14">
+      <c r="F27" s="13">
         <f>SUM(F19:F26)</f>
         <v>41</v>
       </c>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B30" s="10" t="s">
+      <c r="B30" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="10"/>
+      <c r="C30" s="32"/>
+      <c r="D30" s="32"/>
+      <c r="E30" s="32"/>
+      <c r="F30" s="32"/>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
+      <c r="B31" s="32"/>
+      <c r="C31" s="32"/>
+      <c r="D31" s="32"/>
+      <c r="E31" s="32"/>
+      <c r="F31" s="32"/>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B33" s="5" t="s">
@@ -1417,7 +1413,7 @@
       <c r="E34" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="F34" s="15">
+      <c r="F34" s="14">
         <v>8</v>
       </c>
     </row>
@@ -1425,14 +1421,14 @@
       <c r="B35" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C35" s="18" t="s">
+      <c r="C35" s="7" t="s">
         <v>43</v>
       </c>
       <c r="D35" s="7"/>
       <c r="E35" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F35" s="15">
+      <c r="F35" s="14">
         <v>1</v>
       </c>
     </row>
@@ -1440,14 +1436,14 @@
       <c r="B36" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C36" s="11" t="s">
+      <c r="C36" s="10" t="s">
         <v>44</v>
       </c>
       <c r="D36" s="7"/>
       <c r="E36" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F36" s="15">
+      <c r="F36" s="14">
         <v>1</v>
       </c>
     </row>
@@ -1455,29 +1451,29 @@
       <c r="B37" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="C37" s="11" t="s">
+      <c r="C37" s="10" t="s">
         <v>45</v>
       </c>
       <c r="D37" s="7"/>
       <c r="E37" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="F37" s="16">
+      <c r="F37" s="15">
         <v>2</v>
       </c>
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B38" s="12" t="s">
+      <c r="B38" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="C38" s="11" t="s">
+      <c r="C38" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="D38" s="11"/>
+      <c r="D38" s="10"/>
       <c r="E38" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="F38" s="17">
+      <c r="F38" s="16">
         <v>4</v>
       </c>
     </row>
@@ -1485,7 +1481,7 @@
       <c r="D39" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F39" s="14">
+      <c r="F39" s="13">
         <f>SUM(F34:F38)</f>
         <v>16</v>
       </c>
@@ -1511,103 +1507,103 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:19" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="37" t="s">
         <v>53</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
       <c r="J3" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="4" spans="2:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="I4" s="13" t="s">
+      <c r="I4" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="J4" s="25" t="s">
+      <c r="J4" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="K4" s="29" t="s">
+      <c r="K4" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="L4" s="30"/>
-      <c r="M4" s="30"/>
-      <c r="N4" s="30"/>
-      <c r="O4" s="30"/>
-      <c r="P4" s="30"/>
-      <c r="Q4" s="30"/>
-      <c r="R4" s="30"/>
-      <c r="S4" s="31"/>
+      <c r="L4" s="35"/>
+      <c r="M4" s="35"/>
+      <c r="N4" s="35"/>
+      <c r="O4" s="35"/>
+      <c r="P4" s="35"/>
+      <c r="Q4" s="35"/>
+      <c r="R4" s="35"/>
+      <c r="S4" s="36"/>
     </row>
     <row r="5" spans="2:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="I5" s="26" t="s">
+      <c r="I5" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="J5" s="27">
+      <c r="J5" s="22">
         <v>6</v>
       </c>
-      <c r="K5" s="28" t="s">
+      <c r="K5" s="33" t="s">
         <v>73</v>
       </c>
-      <c r="L5" s="28"/>
-      <c r="M5" s="28"/>
-      <c r="N5" s="28"/>
-      <c r="O5" s="28"/>
-      <c r="P5" s="28"/>
-      <c r="Q5" s="28"/>
-      <c r="R5" s="28"/>
-      <c r="S5" s="28"/>
+      <c r="L5" s="33"/>
+      <c r="M5" s="33"/>
+      <c r="N5" s="33"/>
+      <c r="O5" s="33"/>
+      <c r="P5" s="33"/>
+      <c r="Q5" s="33"/>
+      <c r="R5" s="33"/>
+      <c r="S5" s="33"/>
     </row>
     <row r="6" spans="2:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="I6" s="26" t="s">
+      <c r="I6" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="J6" s="27">
+      <c r="J6" s="22">
         <v>10</v>
       </c>
-      <c r="K6" s="28" t="s">
+      <c r="K6" s="33" t="s">
         <v>70</v>
       </c>
-      <c r="L6" s="28"/>
-      <c r="M6" s="28"/>
-      <c r="N6" s="28"/>
-      <c r="O6" s="28"/>
-      <c r="P6" s="28"/>
-      <c r="Q6" s="28"/>
-      <c r="R6" s="28"/>
-      <c r="S6" s="28"/>
+      <c r="L6" s="33"/>
+      <c r="M6" s="33"/>
+      <c r="N6" s="33"/>
+      <c r="O6" s="33"/>
+      <c r="P6" s="33"/>
+      <c r="Q6" s="33"/>
+      <c r="R6" s="33"/>
+      <c r="S6" s="33"/>
     </row>
     <row r="7" spans="2:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="I7" s="26" t="s">
+      <c r="I7" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="J7" s="27">
+      <c r="J7" s="22">
         <v>8</v>
       </c>
-      <c r="K7" s="28" t="s">
+      <c r="K7" s="33" t="s">
         <v>72</v>
       </c>
-      <c r="L7" s="28"/>
-      <c r="M7" s="28"/>
-      <c r="N7" s="28"/>
-      <c r="O7" s="28"/>
-      <c r="P7" s="28"/>
-      <c r="Q7" s="28"/>
-      <c r="R7" s="28"/>
-      <c r="S7" s="28"/>
+      <c r="L7" s="33"/>
+      <c r="M7" s="33"/>
+      <c r="N7" s="33"/>
+      <c r="O7" s="33"/>
+      <c r="P7" s="33"/>
+      <c r="Q7" s="33"/>
+      <c r="R7" s="33"/>
+      <c r="S7" s="33"/>
     </row>
     <row r="9" spans="2:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="17" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1641,7 +1637,7 @@
       <c r="F12" s="7">
         <v>14</v>
       </c>
-      <c r="G12" s="22">
+      <c r="G12" s="19">
         <f>(D12+4*E12+F12)/6</f>
         <v>10.333333333333334</v>
       </c>
@@ -1659,7 +1655,7 @@
       <c r="F13" s="7">
         <v>3</v>
       </c>
-      <c r="G13" s="22">
+      <c r="G13" s="19">
         <f>(D13+4*E13+F13)/6</f>
         <v>2</v>
       </c>
@@ -1677,8 +1673,8 @@
       <c r="F14" s="7">
         <v>6</v>
       </c>
-      <c r="G14" s="22">
-        <f t="shared" ref="G13:G15" si="0">(D14+4*E14+F14)/6</f>
+      <c r="G14" s="19">
+        <f t="shared" ref="G14" si="0">(D14+4*E14+F14)/6</f>
         <v>4.166666666666667</v>
       </c>
     </row>
@@ -1695,7 +1691,7 @@
       <c r="F15" s="7">
         <v>4</v>
       </c>
-      <c r="G15" s="22">
+      <c r="G15" s="19">
         <f>(D15+4*E15+F15)/6</f>
         <v>2.1666666666666665</v>
       </c>
@@ -1713,19 +1709,19 @@
       <c r="F16" s="7">
         <v>2</v>
       </c>
-      <c r="G16" s="22">
+      <c r="G16" s="19">
         <f>(D16+4*E16+F16)/6</f>
         <v>1.0833333333333333</v>
       </c>
     </row>
     <row r="17" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C17" s="21" t="s">
+      <c r="C17" s="18" t="s">
         <v>61</v>
       </c>
       <c r="D17" s="7"/>
       <c r="E17" s="7"/>
       <c r="F17" s="7"/>
-      <c r="G17" s="23">
+      <c r="G17" s="20">
         <f>SUM(G12:G16)</f>
         <v>19.75</v>
       </c>
@@ -1760,7 +1756,7 @@
       <c r="F21" s="7">
         <v>4</v>
       </c>
-      <c r="G21" s="22">
+      <c r="G21" s="19">
         <f>(D21+4*E21+F21)/6</f>
         <v>2.1666666666666665</v>
       </c>
@@ -1778,7 +1774,7 @@
       <c r="F22" s="7">
         <v>5</v>
       </c>
-      <c r="G22" s="22">
+      <c r="G22" s="19">
         <f>(D22+4*E22+F22)/6</f>
         <v>3.1666666666666665</v>
       </c>
@@ -1796,7 +1792,7 @@
       <c r="F23" s="7">
         <v>16</v>
       </c>
-      <c r="G23" s="22">
+      <c r="G23" s="19">
         <f t="shared" ref="G23" si="1">(D23+4*E23+F23)/6</f>
         <v>12.333333333333334</v>
       </c>
@@ -1814,7 +1810,7 @@
       <c r="F24" s="7">
         <v>9</v>
       </c>
-      <c r="G24" s="22">
+      <c r="G24" s="19">
         <f>(D24+4*E24+F24)/6</f>
         <v>6.166666666666667</v>
       </c>
@@ -1832,7 +1828,7 @@
       <c r="F25" s="7">
         <v>12</v>
       </c>
-      <c r="G25" s="22">
+      <c r="G25" s="19">
         <f>(D25+4*E25+F25)/6</f>
         <v>8.3333333333333339</v>
       </c>
@@ -1850,7 +1846,7 @@
       <c r="F26" s="7">
         <v>6</v>
       </c>
-      <c r="G26" s="22">
+      <c r="G26" s="19">
         <f>(D26+4*E26+F26)/6</f>
         <v>4.166666666666667</v>
       </c>
@@ -1868,7 +1864,7 @@
       <c r="F27" s="7">
         <v>6</v>
       </c>
-      <c r="G27" s="22">
+      <c r="G27" s="19">
         <f>(D27+4*E27+F27)/6</f>
         <v>4.166666666666667</v>
       </c>
@@ -1886,19 +1882,19 @@
       <c r="F28" s="7">
         <v>3</v>
       </c>
-      <c r="G28" s="22">
+      <c r="G28" s="19">
         <f t="shared" ref="G28" si="2">(D28+4*E28+F28)/6</f>
         <v>2</v>
       </c>
     </row>
     <row r="29" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C29" s="21" t="s">
+      <c r="C29" s="18" t="s">
         <v>76</v>
       </c>
       <c r="D29" s="7"/>
       <c r="E29" s="7"/>
       <c r="F29" s="7"/>
-      <c r="G29" s="23">
+      <c r="G29" s="20">
         <f>SUM(G21:G28)</f>
         <v>42.5</v>
       </c>
@@ -1933,7 +1929,7 @@
       <c r="F33" s="7">
         <v>12</v>
       </c>
-      <c r="G33" s="22">
+      <c r="G33" s="19">
         <f>(D33+4*E33+F33)/6</f>
         <v>8.3333333333333339</v>
       </c>
@@ -1951,7 +1947,7 @@
       <c r="F34" s="7">
         <v>2</v>
       </c>
-      <c r="G34" s="22">
+      <c r="G34" s="19">
         <f>(D34+4*E34+F34)/6</f>
         <v>1.0833333333333333</v>
       </c>
@@ -1969,7 +1965,7 @@
       <c r="F35" s="7">
         <v>2</v>
       </c>
-      <c r="G35" s="22">
+      <c r="G35" s="19">
         <f t="shared" ref="G35" si="3">(D35+4*E35+F35)/6</f>
         <v>1.0833333333333333</v>
       </c>
@@ -1987,7 +1983,7 @@
       <c r="F36" s="7">
         <v>3</v>
       </c>
-      <c r="G36" s="22">
+      <c r="G36" s="19">
         <f>(D36+4*E36+F36)/6</f>
         <v>2.0833333333333335</v>
       </c>
@@ -2005,28 +2001,28 @@
       <c r="F37" s="7">
         <v>6</v>
       </c>
-      <c r="G37" s="22">
+      <c r="G37" s="19">
         <f>(D37+4*E37+F37)/6</f>
         <v>4.166666666666667</v>
       </c>
     </row>
     <row r="38" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C38" s="21" t="s">
+      <c r="C38" s="18" t="s">
         <v>80</v>
       </c>
       <c r="D38" s="7"/>
       <c r="E38" s="7"/>
       <c r="F38" s="7"/>
-      <c r="G38" s="23">
+      <c r="G38" s="20">
         <f>SUM(G33:G37)</f>
         <v>16.750000000000004</v>
       </c>
     </row>
     <row r="39" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="G39" s="32"/>
+      <c r="G39" s="24"/>
     </row>
     <row r="40" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="G40" s="32"/>
+      <c r="G40" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2049,62 +2045,62 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="C3" s="37" t="s">
+      <c r="C3" s="38" t="s">
         <v>81</v>
       </c>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
     </row>
     <row r="4" spans="3:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="38" t="s">
+      <c r="C4" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="D4" s="39" t="s">
+      <c r="D4" s="34" t="s">
         <v>87</v>
       </c>
-      <c r="E4" s="40"/>
+      <c r="E4" s="36"/>
       <c r="F4" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="5" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C5" s="33" t="s">
+      <c r="C5" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="34" t="s">
         <v>91</v>
       </c>
-      <c r="E5" s="31"/>
+      <c r="E5" s="36"/>
       <c r="F5" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="6" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C6" s="26" t="s">
+      <c r="C6" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="D6" s="35" t="s">
+      <c r="D6" s="39" t="s">
         <v>85</v>
       </c>
-      <c r="E6" s="36"/>
+      <c r="E6" s="40"/>
     </row>
     <row r="7" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C7" s="26" t="s">
+      <c r="C7" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="D7" s="35">
+      <c r="D7" s="39">
         <v>24</v>
       </c>
-      <c r="E7" s="36"/>
+      <c r="E7" s="40"/>
     </row>
     <row r="8" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C8" s="26" t="s">
+      <c r="C8" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="D8" s="34" t="s">
+      <c r="D8" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="E8" s="34"/>
+      <c r="E8" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2123,135 +2119,132 @@
   <dimension ref="B4:K19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="9.140625" style="24"/>
-    <col min="4" max="4" width="11.7109375" style="24" customWidth="1"/>
-    <col min="5" max="5" width="12.42578125" style="24" customWidth="1"/>
-    <col min="6" max="10" width="9.140625" style="24"/>
-    <col min="11" max="11" width="39.140625" style="24" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="24"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" customWidth="1"/>
+    <col min="11" max="11" width="39.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:11" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="B4" s="41" t="s">
+    <row r="4" spans="2:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B4" s="45" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="5" spans="2:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B5" s="42" t="s">
+      <c r="B5" s="26" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B6" s="24" t="s">
+    <row r="6" spans="2:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B6" s="46" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="8" spans="2:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B8" s="51" t="s">
+      <c r="B8" s="31" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="9" spans="2:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="51" t="s">
+      <c r="B9" s="31" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="13" spans="2:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B13" s="43" t="s">
+      <c r="B13" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="C13" s="43"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="43"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="43"/>
-      <c r="H13" s="43"/>
-      <c r="I13" s="43"/>
-      <c r="J13" s="43"/>
-      <c r="K13" s="43"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="27"/>
+      <c r="J13" s="27"/>
+      <c r="K13" s="27"/>
     </row>
     <row r="14" spans="2:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B14" s="44" t="s">
+      <c r="B14" s="42" t="s">
         <v>98</v>
       </c>
-      <c r="C14" s="44"/>
-      <c r="D14" s="44"/>
-      <c r="E14" s="45" t="s">
+      <c r="C14" s="42"/>
+      <c r="D14" s="42"/>
+      <c r="E14" s="28" t="s">
         <v>87</v>
       </c>
-      <c r="F14" s="46" t="s">
+      <c r="F14" s="44" t="s">
         <v>100</v>
       </c>
-      <c r="G14" s="46"/>
-      <c r="H14" s="46"/>
-      <c r="I14" s="46"/>
-      <c r="J14" s="46"/>
-      <c r="K14" s="46"/>
+      <c r="G14" s="44"/>
+      <c r="H14" s="44"/>
+      <c r="I14" s="44"/>
+      <c r="J14" s="44"/>
+      <c r="K14" s="44"/>
     </row>
     <row r="15" spans="2:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B15" s="47" t="s">
+      <c r="B15" s="43" t="s">
         <v>104</v>
       </c>
-      <c r="C15" s="47"/>
-      <c r="D15" s="47"/>
-      <c r="E15" s="48" t="s">
+      <c r="C15" s="43"/>
+      <c r="D15" s="43"/>
+      <c r="E15" s="29" t="s">
         <v>101</v>
       </c>
-      <c r="F15" s="49" t="s">
+      <c r="F15" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="G15" s="49"/>
-      <c r="H15" s="49"/>
-      <c r="I15" s="49"/>
-      <c r="J15" s="49"/>
-      <c r="K15" s="49"/>
+      <c r="G15" s="41"/>
+      <c r="H15" s="41"/>
+      <c r="I15" s="41"/>
+      <c r="J15" s="41"/>
+      <c r="K15" s="41"/>
     </row>
     <row r="16" spans="2:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B16" s="47" t="s">
+      <c r="B16" s="43" t="s">
         <v>105</v>
       </c>
-      <c r="C16" s="47"/>
-      <c r="D16" s="47"/>
-      <c r="E16" s="48" t="s">
+      <c r="C16" s="43"/>
+      <c r="D16" s="43"/>
+      <c r="E16" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="F16" s="49" t="s">
+      <c r="F16" s="41" t="s">
         <v>108</v>
       </c>
-      <c r="G16" s="49"/>
-      <c r="H16" s="49"/>
-      <c r="I16" s="49"/>
-      <c r="J16" s="49"/>
-      <c r="K16" s="49"/>
+      <c r="G16" s="41"/>
+      <c r="H16" s="41"/>
+      <c r="I16" s="41"/>
+      <c r="J16" s="41"/>
+      <c r="K16" s="41"/>
     </row>
     <row r="17" spans="2:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B17" s="47" t="s">
+      <c r="B17" s="43" t="s">
         <v>106</v>
       </c>
-      <c r="C17" s="47"/>
-      <c r="D17" s="47"/>
-      <c r="E17" s="48" t="s">
+      <c r="C17" s="43"/>
+      <c r="D17" s="43"/>
+      <c r="E17" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="F17" s="49" t="s">
+      <c r="F17" s="41" t="s">
         <v>99</v>
       </c>
-      <c r="G17" s="49"/>
-      <c r="H17" s="49"/>
-      <c r="I17" s="49"/>
-      <c r="J17" s="49"/>
-      <c r="K17" s="49"/>
+      <c r="G17" s="41"/>
+      <c r="H17" s="41"/>
+      <c r="I17" s="41"/>
+      <c r="J17" s="41"/>
+      <c r="K17" s="41"/>
     </row>
     <row r="19" spans="2:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B19" s="24" t="s">
+      <c r="B19" s="46" t="s">
         <v>109</v>
       </c>
-      <c r="F19" s="50"/>
-      <c r="G19" s="50"/>
-      <c r="H19" s="50"/>
-      <c r="I19" s="50"/>
-      <c r="J19" s="50"/>
-      <c r="K19" s="50"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="30"/>
+      <c r="I19" s="30"/>
+      <c r="J19" s="30"/>
+      <c r="K19" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>